<commit_message>
dashboard updated and MVPF alternatives table added
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56EA14A-4595-F040-822C-8FF4A1E80F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14FE762-6AF7-814F-BC64-75959BABEE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -498,18 +498,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -814,22 +815,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T24"/>
+  <dimension ref="A1:T26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="81.5" customWidth="1"/>
+    <col min="3" max="3" width="59.83203125" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.33203125" customWidth="1"/>
     <col min="8" max="8" width="43.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="53.6640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="72.1640625" bestFit="1" customWidth="1"/>
@@ -897,31 +898,31 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="I2" s="8"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="O2" s="5" t="s">
+      <c r="I2" s="6"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+      <c r="O2" s="3" t="s">
         <v>21</v>
       </c>
     </row>
@@ -947,19 +948,19 @@
       <c r="H3" t="s">
         <v>102</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="7">
         <v>973000</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="7">
         <v>100000</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="7">
         <v>973000</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="8">
         <v>294728</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="7">
         <v>10000000</v>
       </c>
       <c r="O3" t="s">
@@ -982,11 +983,11 @@
       <c r="D4" t="s">
         <v>120</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="3"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="7"/>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1010,17 +1011,17 @@
       <c r="H5" t="s">
         <v>108</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="7">
         <v>875000</v>
       </c>
-      <c r="J5" s="3">
+      <c r="J5" s="7">
         <v>500000</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="7">
         <v>875000</v>
       </c>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3">
+      <c r="L5" s="7"/>
+      <c r="M5" s="7">
         <v>1200000</v>
       </c>
       <c r="O5" t="s">
@@ -1058,7 +1059,11 @@
       <c r="E6" t="s">
         <v>31</v>
       </c>
-      <c r="I6" s="3"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1079,20 +1084,20 @@
       <c r="F7" t="s">
         <v>118</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <v>2017</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="7">
         <v>75000</v>
       </c>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3">
+      <c r="J7" s="7"/>
+      <c r="K7" s="7">
         <v>133685</v>
       </c>
-      <c r="L7" s="3">
+      <c r="L7" s="7">
         <v>75000</v>
       </c>
-      <c r="M7" s="3"/>
+      <c r="M7" s="7"/>
       <c r="O7" t="s">
         <v>28</v>
       </c>
@@ -1112,31 +1117,31 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:20" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:20" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="O8" s="5" t="s">
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="O8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="Q8" s="5" t="s">
+      <c r="Q8" s="3" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1162,17 +1167,17 @@
       <c r="G9">
         <v>2018</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="7">
         <v>3677</v>
       </c>
-      <c r="J9" s="2">
+      <c r="J9" s="7">
         <v>1710</v>
       </c>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2">
+      <c r="K9" s="7"/>
+      <c r="L9" s="7">
         <v>3677</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="7">
         <v>5623</v>
       </c>
       <c r="O9" t="s">
@@ -1201,15 +1206,15 @@
       <c r="F10" t="s">
         <v>35</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="7">
         <v>60.37</v>
       </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2">
+      <c r="J10" s="7"/>
+      <c r="K10" s="7">
         <v>60.37</v>
       </c>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
       <c r="O10" t="s">
         <v>28</v>
       </c>
@@ -1242,15 +1247,15 @@
       <c r="F11" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="7">
         <v>0.61</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="7">
         <v>0.61</v>
       </c>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11">
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7">
         <v>0.71</v>
       </c>
       <c r="O11" t="s">
@@ -1291,20 +1296,20 @@
       <c r="G12">
         <v>2011</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="7">
         <v>11</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="7">
         <v>11</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="7">
         <v>33</v>
       </c>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
       <c r="O12" t="s">
         <v>28</v>
       </c>
@@ -1334,15 +1339,15 @@
       <c r="F13" t="s">
         <v>35</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="7">
         <v>4.9400000000000004</v>
       </c>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2">
+      <c r="J13" s="7"/>
+      <c r="K13" s="7">
         <v>4.9400000000000004</v>
       </c>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
       <c r="O13" t="s">
         <v>28</v>
       </c>
@@ -1378,13 +1383,13 @@
       <c r="H14" t="s">
         <v>65</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="7">
         <v>99.44</v>
       </c>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
       <c r="O14" t="s">
         <v>28</v>
       </c>
@@ -1411,15 +1416,15 @@
       <c r="G15">
         <v>2022</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="7">
         <v>11</v>
       </c>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2">
+      <c r="J15" s="7"/>
+      <c r="K15" s="7">
         <v>11</v>
       </c>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="7"/>
       <c r="O15" t="s">
         <v>28</v>
       </c>
@@ -1455,15 +1460,15 @@
       <c r="H16" t="s">
         <v>73</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="7">
         <v>249634</v>
       </c>
-      <c r="J16">
+      <c r="J16" s="7">
         <v>178920</v>
       </c>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16">
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7">
         <v>249634</v>
       </c>
       <c r="O16" t="s">
@@ -1498,15 +1503,15 @@
       <c r="G17">
         <v>2017</v>
       </c>
-      <c r="I17" s="3">
+      <c r="I17" s="7">
         <v>130</v>
       </c>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2">
+      <c r="J17" s="7"/>
+      <c r="K17" s="7">
         <v>130</v>
       </c>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
       <c r="O17" t="s">
         <v>21</v>
       </c>
@@ -1542,20 +1547,20 @@
       <c r="G18">
         <v>2015</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="I18" s="3">
+      <c r="I18" s="7">
         <v>50</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="7">
         <v>25</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="7">
         <v>50</v>
       </c>
-      <c r="L18" s="2"/>
-      <c r="M18">
+      <c r="L18" s="7"/>
+      <c r="M18" s="7">
         <v>100</v>
       </c>
       <c r="O18" t="s">
@@ -1590,15 +1595,15 @@
       <c r="G19">
         <v>2018</v>
       </c>
-      <c r="I19" s="3">
+      <c r="I19" s="7">
         <v>300</v>
       </c>
-      <c r="J19">
+      <c r="J19" s="7">
         <v>200</v>
       </c>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19">
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7">
         <v>400</v>
       </c>
       <c r="O19" t="s">
@@ -1636,18 +1641,18 @@
       <c r="G20">
         <v>2018</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="I20" s="3">
+      <c r="I20" s="7">
         <v>448677628</v>
       </c>
-      <c r="J20">
+      <c r="J20" s="7">
         <v>448677628</v>
       </c>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
       <c r="O20" t="s">
         <v>28</v>
       </c>
@@ -1677,13 +1682,13 @@
       <c r="G21">
         <v>2018</v>
       </c>
-      <c r="I21" s="3">
+      <c r="I21" s="7">
         <v>33945</v>
       </c>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
@@ -1704,9 +1709,13 @@
       <c r="G22">
         <v>2018</v>
       </c>
-      <c r="I22" s="3">
+      <c r="I22" s="7">
         <v>5171000</v>
       </c>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
@@ -1715,7 +1724,7 @@
       <c r="B23" t="s">
         <v>96</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>130</v>
       </c>
       <c r="E23" t="s">
@@ -1727,12 +1736,34 @@
       <c r="G23">
         <v>2018</v>
       </c>
-      <c r="I23" s="3">
+      <c r="I23" s="7">
         <v>100000</v>
       </c>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="I24" s="3"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated some terms due to new LoS assumptions
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56EA14A-4595-F040-822C-8FF4A1E80F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F644ED30-C8C0-F946-A689-9B96AB765409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -438,7 +438,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
@@ -498,7 +499,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -510,6 +511,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1456,15 +1458,12 @@
         <v>73</v>
       </c>
       <c r="I16" s="3">
-        <v>249634</v>
-      </c>
-      <c r="J16">
-        <v>178920</v>
+        <v>295275</v>
       </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
-      <c r="M16">
-        <v>249634</v>
+      <c r="M16" s="9">
+        <v>295275</v>
       </c>
       <c r="O16" t="s">
         <v>28</v>

</xml_diff>

<commit_message>
dashboard and table changes
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14FE762-6AF7-814F-BC64-75959BABEE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B86A90-B744-F845-96BC-38C1D13BB9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -441,7 +441,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -477,6 +477,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -495,10 +503,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -511,8 +520,10 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -825,7 +836,7 @@
     <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.33203125" customWidth="1"/>
-    <col min="8" max="8" width="43.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.33203125" customWidth="1"/>
     <col min="9" max="9" width="19.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
@@ -948,8 +959,8 @@
       <c r="H3" t="s">
         <v>102</v>
       </c>
-      <c r="I3" s="7">
-        <v>973000</v>
+      <c r="I3" s="8">
+        <v>294728</v>
       </c>
       <c r="J3" s="7">
         <v>100000</v>
@@ -966,7 +977,7 @@
       <c r="O3" t="s">
         <v>21</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="10" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1012,17 +1023,17 @@
         <v>108</v>
       </c>
       <c r="I5" s="7">
-        <v>875000</v>
+        <v>16785</v>
       </c>
       <c r="J5" s="7">
-        <v>500000</v>
+        <v>9377</v>
       </c>
       <c r="K5" s="7">
-        <v>875000</v>
+        <v>16785</v>
       </c>
       <c r="L5" s="7"/>
       <c r="M5" s="7">
-        <v>1200000</v>
+        <v>37518</v>
       </c>
       <c r="O5" t="s">
         <v>21</v>
@@ -1107,13 +1118,13 @@
       <c r="Q7" t="s">
         <v>111</v>
       </c>
-      <c r="R7" t="s">
+      <c r="R7" s="10" t="s">
         <v>112</v>
       </c>
       <c r="S7" t="s">
         <v>113</v>
       </c>
-      <c r="T7" t="s">
+      <c r="T7" s="10" t="s">
         <v>109</v>
       </c>
     </row>
@@ -1766,6 +1777,11 @@
       <c r="M26" s="7"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="R7" r:id="rId1" xr:uid="{DB52D8D2-D913-6047-A2C0-C19889E9CABC}"/>
+    <hyperlink ref="T7" r:id="rId2" xr:uid="{99E21AE3-A092-4248-BD86-FB2A04B383D0}"/>
+    <hyperlink ref="R3" r:id="rId3" xr:uid="{59664F8A-ED6E-714E-A53D-A9C25DDCDE66}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add value for court appearance from nudge paper
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F70A88-DBF9-3945-B82D-C887358E98FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A49AAD6-7B03-CF42-9CDD-DED41A7C8B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3200" yWindow="760" windowWidth="26200" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline components " sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="151">
   <si>
     <t>row_var</t>
   </si>
@@ -434,9 +434,6 @@
     <t>2018 Annual Appropriations</t>
   </si>
   <si>
-    <t xml:space="preserve">formula </t>
-  </si>
-  <si>
     <t>Min alternative</t>
   </si>
   <si>
@@ -483,6 +480,15 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Numerator Additive component Name</t>
+  </si>
+  <si>
+    <t>component value</t>
+  </si>
+  <si>
+    <t>Denominator Additive component Name</t>
   </si>
 </sst>
 </file>
@@ -565,7 +571,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -579,10 +585,9 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -920,7 +925,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -938,10 +943,10 @@
         <v>111</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>11</v>
@@ -959,40 +964,46 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+    <row r="2" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="C2" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="C2" s="14" t="s">
+      <c r="D2" s="13">
+        <v>1</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>137</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="G2" s="13">
+        <v>2020</v>
+      </c>
+      <c r="H2" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="D2" s="14">
-        <v>1</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>138</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" s="14" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="14" t="s">
+      <c r="I2" s="13">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>135</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="D3" s="14">
+      <c r="B3" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" s="11">
         <v>1</v>
       </c>
     </row>
@@ -1001,16 +1012,16 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" t="s">
         <v>35</v>
@@ -1036,7 +1047,7 @@
         <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C5" t="s">
         <v>66</v>
@@ -1070,10 +1081,10 @@
         <v>69</v>
       </c>
       <c r="B6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1108,7 +1119,7 @@
         <v>85</v>
       </c>
       <c r="B7" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C7" t="s">
         <v>86</v>
@@ -1149,7 +1160,7 @@
         <v>89</v>
       </c>
       <c r="B8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C8" t="s">
         <v>90</v>
@@ -1198,7 +1209,7 @@
         <v>95</v>
       </c>
       <c r="F9" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G9">
         <v>2018</v>
@@ -1226,7 +1237,7 @@
         <v>95</v>
       </c>
       <c r="F10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G10">
         <v>2018</v>
@@ -1252,10 +1263,10 @@
         <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I11" s="3">
         <v>0.7</v>
@@ -1278,10 +1289,10 @@
         <v>41</v>
       </c>
       <c r="F12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G12" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I12" s="3">
         <v>70</v>
@@ -1310,12 +1321,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCEB78A-8117-3143-B4E8-94B34C4CEAC6}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="31.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>132</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1362,7 +1388,7 @@
         <v>111</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>8</v>
@@ -1371,7 +1397,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>11</v>
@@ -1389,28 +1415,28 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:19" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" t="s">
         <v>30</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" t="s">
         <v>31</v>
       </c>
-      <c r="I2" s="12"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="P2" s="11" t="s">
+      <c r="I2" s="3"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="P2" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding crime detention selected_value
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A49AAD6-7B03-CF42-9CDD-DED41A7C8B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93AF519A-1F2D-6B49-8894-C1E5E179B313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3200" yWindow="760" windowWidth="26200" windowHeight="14500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-2140" yWindow="-27360" windowWidth="32280" windowHeight="16500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline components " sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="151">
   <si>
     <t>row_var</t>
   </si>
@@ -473,9 +473,6 @@
     <t>baseline (1) /alternative</t>
   </si>
   <si>
-    <t>Incapacitation and deterrance crime effects of detention, valued by RHV</t>
-  </si>
-  <si>
     <t>Wrongful death damages Social cost of detainment (remove wtp for a human life)</t>
   </si>
   <si>
@@ -489,6 +486,9 @@
   </si>
   <si>
     <t>Denominator Additive component Name</t>
+  </si>
+  <si>
+    <t>Incapacitation and deterrance crime effects of detention</t>
   </si>
 </sst>
 </file>
@@ -544,18 +544,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -571,7 +565,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -585,9 +579,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -964,47 +956,56 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>140</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" t="s">
         <v>134</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" t="s">
         <v>141</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" t="s">
         <v>137</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" t="s">
         <v>115</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2">
         <v>2020</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" t="s">
         <v>142</v>
       </c>
-      <c r="I2" s="13">
+      <c r="I2">
         <v>12.6</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" t="s">
         <v>134</v>
       </c>
-      <c r="C3" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="D3" s="11">
+      <c r="C3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D3">
         <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F3" t="s">
+        <v>115</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
@@ -1015,7 +1016,7 @@
         <v>134</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1155,7 +1156,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>89</v>
       </c>
@@ -1209,7 +1210,7 @@
         <v>95</v>
       </c>
       <c r="F9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G9">
         <v>2018</v>
@@ -1237,7 +1238,7 @@
         <v>95</v>
       </c>
       <c r="F10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G10">
         <v>2018</v>
@@ -1263,10 +1264,10 @@
         <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G11" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I11" s="3">
         <v>0.7</v>
@@ -1289,10 +1290,10 @@
         <v>41</v>
       </c>
       <c r="F12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G12" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I12" s="3">
         <v>70</v>
@@ -1329,19 +1330,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="12" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="11" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>149</v>
+      <c r="B7" s="11" t="s">
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changed value to society component reference dollar amounts
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93AF519A-1F2D-6B49-8894-C1E5E179B313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA1056A7-0564-5A48-A2AD-070496E21CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2140" yWindow="-27360" windowWidth="32280" windowHeight="16500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline components " sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="156">
   <si>
     <t>row_var</t>
   </si>
@@ -488,7 +488,22 @@
     <t>Denominator Additive component Name</t>
   </si>
   <si>
-    <t>Incapacitation and deterrance crime effects of detention</t>
+    <t>Hofflander ( ): Loss of Income Due to Wrongful Death: A Method of Measurement.Insurance Law Journal 1965 Ins. L.J. (1965)  LibGuide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lewbel (2003)l: Calculating compensation in cases of wrongful death. Journal of Econometrics 113, pp 115-128 </t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/pii/S0304407602001690#SEC2</t>
+  </si>
+  <si>
+    <t>US statistics from https://www.scheuermanlaw.com/wrongful-death-settlement-calculator/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incapacitation and deterrance crime effects of detention measured by Monetary D- bonds </t>
+  </si>
+  <si>
+    <t>D-bond values selected for felony charges</t>
   </si>
 </sst>
 </file>
@@ -499,7 +514,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -543,6 +558,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -565,7 +586,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -580,6 +601,10 @@
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -885,12 +910,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018C5E1B-70FC-CE48-BD0C-84D5CA275194}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="61" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="77.6640625" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" bestFit="1" customWidth="1"/>
@@ -993,7 +1018,7 @@
         <v>134</v>
       </c>
       <c r="C3" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1004,18 +1029,39 @@
       <c r="F3" t="s">
         <v>115</v>
       </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I3" s="3">
+        <v>75000</v>
+      </c>
+      <c r="J3" s="3">
+        <v>133685</v>
+      </c>
+      <c r="K3" s="3">
+        <v>75000</v>
+      </c>
+      <c r="L3" t="s">
+        <v>155</v>
+      </c>
+      <c r="M3" t="s">
+        <v>108</v>
+      </c>
+      <c r="N3" t="s">
+        <v>109</v>
+      </c>
+      <c r="O3" t="s">
+        <v>110</v>
+      </c>
+      <c r="P3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>134</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="13" t="s">
         <v>145</v>
       </c>
       <c r="D4">
@@ -1031,64 +1077,45 @@
         <v>99</v>
       </c>
       <c r="I4" s="3">
-        <v>973000</v>
+        <v>294728</v>
       </c>
       <c r="J4" s="3">
         <v>100000</v>
       </c>
       <c r="K4" s="3">
-        <v>10000000</v>
+        <v>300000</v>
+      </c>
+      <c r="M4" s="12" t="s">
+        <v>151</v>
       </c>
       <c r="N4" t="s">
-        <v>98</v>
+        <v>152</v>
+      </c>
+      <c r="O4" t="s">
+        <v>150</v>
+      </c>
+      <c r="P4" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G5">
-        <v>2022</v>
-      </c>
-      <c r="I5" s="3">
-        <v>11</v>
-      </c>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="M5" t="s">
-        <v>67</v>
-      </c>
-      <c r="N5" t="s">
-        <v>68</v>
-      </c>
+      <c r="C5" s="7"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
         <v>135</v>
       </c>
       <c r="C6" t="s">
-        <v>143</v>
+        <v>66</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="s">
         <v>63</v>
@@ -1097,17 +1124,13 @@
         <v>35</v>
       </c>
       <c r="G6">
-        <v>2021</v>
-      </c>
-      <c r="H6" t="s">
-        <v>72</v>
+        <v>2022</v>
       </c>
       <c r="I6" s="3">
-        <v>295275</v>
-      </c>
-      <c r="K6" s="9">
-        <v>295275</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
       <c r="M6" t="s">
         <v>67</v>
       </c>
@@ -1117,60 +1140,57 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7">
+        <v>2021</v>
+      </c>
+      <c r="H7" t="s">
+        <v>72</v>
+      </c>
+      <c r="I7" s="3">
+        <v>295275</v>
+      </c>
+      <c r="K7" s="9">
+        <v>295275</v>
+      </c>
+      <c r="M7" t="s">
+        <v>67</v>
+      </c>
+      <c r="N7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>85</v>
-      </c>
-      <c r="B7" t="s">
-        <v>136</v>
-      </c>
-      <c r="C7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7">
-        <v>3</v>
-      </c>
-      <c r="E7" t="s">
-        <v>125</v>
-      </c>
-      <c r="F7" t="s">
-        <v>115</v>
-      </c>
-      <c r="G7">
-        <v>2018</v>
-      </c>
-      <c r="I7" s="3">
-        <v>300</v>
-      </c>
-      <c r="J7">
-        <v>200</v>
-      </c>
-      <c r="K7">
-        <v>400</v>
-      </c>
-      <c r="L7" t="s">
-        <v>87</v>
-      </c>
-      <c r="M7" t="s">
-        <v>88</v>
-      </c>
-      <c r="N7" s="10" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>89</v>
       </c>
       <c r="B8" t="s">
         <v>136</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="s">
-        <v>91</v>
+        <v>125</v>
       </c>
       <c r="F8" t="s">
         <v>115</v>
@@ -1178,58 +1198,71 @@
       <c r="G8">
         <v>2018</v>
       </c>
-      <c r="H8" s="7"/>
       <c r="I8" s="3">
-        <v>448677628</v>
+        <v>300</v>
       </c>
       <c r="J8">
-        <v>448677628</v>
-      </c>
-      <c r="K8" s="2"/>
+        <v>200</v>
+      </c>
+      <c r="K8">
+        <v>400</v>
+      </c>
+      <c r="L8" t="s">
+        <v>87</v>
+      </c>
       <c r="M8" t="s">
-        <v>131</v>
+        <v>88</v>
       </c>
       <c r="N8" s="10" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B9" t="s">
-        <v>93</v>
+        <v>136</v>
       </c>
       <c r="C9" t="s">
-        <v>94</v>
-      </c>
-      <c r="D9" t="s">
-        <v>117</v>
+        <v>90</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F9" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="G9">
         <v>2018</v>
       </c>
+      <c r="H9" s="7"/>
       <c r="I9" s="3">
-        <v>33945</v>
-      </c>
-      <c r="J9" s="2"/>
+        <v>448677628</v>
+      </c>
+      <c r="J9">
+        <v>448677628</v>
+      </c>
       <c r="K9" s="2"/>
+      <c r="M9" t="s">
+        <v>131</v>
+      </c>
+      <c r="N9" s="10" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B10" t="s">
         <v>93</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D10" t="s">
         <v>117</v>
@@ -1244,50 +1277,52 @@
         <v>2018</v>
       </c>
       <c r="I10" s="3">
-        <v>5171000</v>
-      </c>
+        <v>33945</v>
+      </c>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="B11" t="s">
         <v>93</v>
       </c>
       <c r="C11" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="D11" t="s">
         <v>117</v>
       </c>
       <c r="E11" t="s">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="F11" t="s">
         <v>146</v>
       </c>
-      <c r="G11" t="s">
-        <v>146</v>
+      <c r="G11">
+        <v>2018</v>
       </c>
       <c r="I11" s="3">
-        <v>0.7</v>
+        <v>5171000</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>119</v>
       </c>
       <c r="B12" t="s">
         <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>118</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>117</v>
       </c>
       <c r="E12" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F12" t="s">
         <v>146</v>
@@ -1296,25 +1331,51 @@
         <v>146</v>
       </c>
       <c r="I12" s="3">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" t="s">
+        <v>146</v>
+      </c>
+      <c r="G13" t="s">
+        <v>146</v>
+      </c>
+      <c r="I13" s="3">
         <v>70</v>
       </c>
-      <c r="J12" s="2">
+      <c r="J13" s="2">
         <v>60.37</v>
       </c>
-      <c r="K12" s="2"/>
-      <c r="L12" t="s">
+      <c r="K13" s="2"/>
+      <c r="L13" t="s">
         <v>42</v>
       </c>
-      <c r="M12" t="s">
+      <c r="M13" t="s">
         <v>43</v>
       </c>
-      <c r="N12" t="s">
+      <c r="N13" t="s">
         <v>44</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="N7" r:id="rId1" xr:uid="{126C1809-D3C8-9244-9EA2-45648641ED16}"/>
+    <hyperlink ref="N8" r:id="rId1" xr:uid="{126C1809-D3C8-9244-9EA2-45648641ED16}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1836,7 +1897,7 @@
       <c r="O3" t="s">
         <v>21</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3" s="10" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1903,7 +1964,7 @@
       <c r="Q5" t="s">
         <v>101</v>
       </c>
-      <c r="R5" t="s">
+      <c r="R5" s="10" t="s">
         <v>25</v>
       </c>
       <c r="S5" t="s">
@@ -2580,6 +2641,8 @@
   <hyperlinks>
     <hyperlink ref="R19" r:id="rId1" xr:uid="{913DD2C2-09D4-6340-B25B-D342990A3AE8}"/>
     <hyperlink ref="R11" r:id="rId2" xr:uid="{C43FA892-8D61-5549-A0D1-6272414542B3}"/>
+    <hyperlink ref="R5" r:id="rId3" xr:uid="{5D753F69-E906-C04B-9822-C8DAFD369E0A}"/>
+    <hyperlink ref="R3" r:id="rId4" xr:uid="{A8715A40-89FF-2646-97A1-6C834ED4F68F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
New modular code structure (dashboard, calculator, graph, technical modules), parameter mapping table added
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11102"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA962121-4A3E-0B4C-8557-EBAFBEF4823C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F776D7A-CE38-6D41-B105-65AEED820DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline components " sheetId="4" r:id="rId1"/>
-    <sheet name="MVPF calculation" sheetId="2" r:id="rId2"/>
+    <sheet name="mvpf_component_mapping" sheetId="5" r:id="rId2"/>
     <sheet name="CCJ Subset Quantification" sheetId="3" r:id="rId3"/>
     <sheet name="OLD Baseline components" sheetId="1" r:id="rId4"/>
   </sheets>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="169">
   <si>
     <t>row_var</t>
   </si>
@@ -473,21 +473,9 @@
     <t>baseline (1) /alternative</t>
   </si>
   <si>
-    <t>Wrongful death damages Social cost of detainment (remove wtp for a human life)</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
-    <t>Numerator Additive component Name</t>
-  </si>
-  <si>
-    <t>component value</t>
-  </si>
-  <si>
-    <t>Denominator Additive component Name</t>
-  </si>
-  <si>
     <t>Hofflander ( ): Loss of Income Due to Wrongful Death: A Method of Measurement.Insurance Law Journal 1965 Ins. L.J. (1965)  LibGuide</t>
   </si>
   <si>
@@ -500,12 +488,6 @@
     <t>US statistics from https://www.scheuermanlaw.com/wrongful-death-settlement-calculator/</t>
   </si>
   <si>
-    <t xml:space="preserve">Incapacitation and deterrance crime effects of detention measured by Monetary D- bonds </t>
-  </si>
-  <si>
-    <t>D-bond values selected for felony charges</t>
-  </si>
-  <si>
     <t>crime type - felonies selected</t>
   </si>
   <si>
@@ -519,6 +501,48 @@
   </si>
   <si>
     <t>only for violent crimes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incapacitation and deterrance crime effects of detention  </t>
+  </si>
+  <si>
+    <t>Alternatives proven to be ineffecive: D-bond values selected for felony charges</t>
+  </si>
+  <si>
+    <t>Wrongful death damages Social cost of detainment (focusing on economic impact submeasure)</t>
+  </si>
+  <si>
+    <t>baseline</t>
+  </si>
+  <si>
+    <t>no. of criteria</t>
+  </si>
+  <si>
+    <t>govt_refractions</t>
+  </si>
+  <si>
+    <t>govt_health</t>
+  </si>
+  <si>
+    <t>govt_operative</t>
+  </si>
+  <si>
+    <t>soc_community</t>
+  </si>
+  <si>
+    <t>soc_crimeprev</t>
+  </si>
+  <si>
+    <t>soc_court</t>
+  </si>
+  <si>
+    <t>det_rhv</t>
+  </si>
+  <si>
+    <t>det_wtp</t>
+  </si>
+  <si>
+    <t>Scenario</t>
   </si>
 </sst>
 </file>
@@ -601,7 +625,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -615,11 +639,12 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -925,19 +950,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018C5E1B-70FC-CE48-BD0C-84D5CA275194}">
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="77.6640625" customWidth="1"/>
-    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="3" max="3" width="58.1640625" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
     <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.1640625" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.33203125" customWidth="1"/>
     <col min="12" max="12" width="53.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="72.1640625" bestFit="1" customWidth="1"/>
@@ -1033,7 +1058,7 @@
         <v>134</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1048,10 +1073,10 @@
         <v>2018</v>
       </c>
       <c r="H3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I3" s="3">
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="J3" s="3">
         <v>133685</v>
@@ -1060,7 +1085,7 @@
         <v>75000</v>
       </c>
       <c r="L3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M3" t="s">
         <v>108</v>
@@ -1075,15 +1100,15 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>134</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>145</v>
+      <c r="C4" s="12" t="s">
+        <v>157</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1098,7 +1123,7 @@
         <v>2023</v>
       </c>
       <c r="H4" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="I4" s="3">
         <v>294728</v>
@@ -1110,19 +1135,19 @@
         <v>300000</v>
       </c>
       <c r="L4" t="s">
-        <v>158</v>
-      </c>
-      <c r="M4" s="12" t="s">
-        <v>151</v>
+        <v>152</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>147</v>
       </c>
       <c r="N4" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="O4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="P4" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -1133,7 +1158,7 @@
         <v>134</v>
       </c>
       <c r="C5" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1148,7 +1173,7 @@
         <v>2024</v>
       </c>
       <c r="H5" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="I5" s="3">
         <v>875000</v>
@@ -1160,7 +1185,7 @@
         <v>875000</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="M5" t="s">
         <v>100</v>
@@ -1345,7 +1370,7 @@
         <v>95</v>
       </c>
       <c r="F10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G10">
         <v>2018</v>
@@ -1373,7 +1398,7 @@
         <v>95</v>
       </c>
       <c r="F11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G11">
         <v>2018</v>
@@ -1399,10 +1424,10 @@
         <v>31</v>
       </c>
       <c r="F12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I12" s="3">
         <v>0.7</v>
@@ -1425,10 +1450,10 @@
         <v>41</v>
       </c>
       <c r="F13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I13" s="3">
         <v>70</v>
@@ -1445,6 +1470,12 @@
       </c>
       <c r="N13" t="s">
         <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="9:9" x14ac:dyDescent="0.2">
+      <c r="I19">
+        <f>+I9/I10</f>
+        <v>13217.782530564147</v>
       </c>
     </row>
   </sheetData>
@@ -1457,28 +1488,572 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCEB78A-8117-3143-B4E8-94B34C4CEAC6}">
-  <dimension ref="A1:B7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E4AB0FE-E22E-7046-8B42-84C7BB8E6363}">
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="1" max="1" width="17.5" customWidth="1"/>
+    <col min="2" max="9" width="15.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>148</v>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F1" t="s">
+        <v>163</v>
+      </c>
+      <c r="G1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H1" t="s">
+        <v>161</v>
+      </c>
+      <c r="I1" t="s">
+        <v>160</v>
+      </c>
+      <c r="J1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <f>COUNTIF(B2:I2, 1)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <f>COUNTIF(B3:I3, 1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <f>COUNTIF(B4:I4, 1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <f>COUNTIF(B5:I5, 1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <f>COUNTIF(B6:I6, 1)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <f>COUNTIF(B7:I7, 1)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <f>COUNTIF(B8:I8, 1)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <f>COUNTIF(B9:I9, 1)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <f>COUNTIF(B10:I10, 1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <f>COUNTIF(B11:I11, 1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <f>COUNTIF(B12:I12, 1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <f>COUNTIF(B13:I13, 1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <f>COUNTIF(B14:I14, 1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <f>COUNTIF(B15:I15, 1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <f>COUNTIF(B16:I16, 1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <f>COUNTIF(B17:I17, 1)</f>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dashboard fetaure updates, explainer boxes and more
</commit_message>
<xml_diff>
--- a/Data/CCJ_quantified_values.xlsx
+++ b/Data/CCJ_quantified_values.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11012"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/td/PycharmProjects/CCJ/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/larapesceares/CCJ/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F776D7A-CE38-6D41-B105-65AEED820DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F730FF-DE0A-3446-A64B-28624B00AE94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Baseline components " sheetId="4" r:id="rId1"/>
-    <sheet name="mvpf_component_mapping" sheetId="5" r:id="rId2"/>
-    <sheet name="CCJ Subset Quantification" sheetId="3" r:id="rId3"/>
-    <sheet name="OLD Baseline components" sheetId="1" r:id="rId4"/>
+    <sheet name="CCJ Subset Quantification" sheetId="3" r:id="rId2"/>
+    <sheet name="OLD Baseline components" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="158">
   <si>
     <t>row_var</t>
   </si>
@@ -488,6 +487,12 @@
     <t>US statistics from https://www.scheuermanlaw.com/wrongful-death-settlement-calculator/</t>
   </si>
   <si>
+    <t xml:space="preserve">Incapacitation and deterrance crime effects of detention measured by Monetary D- bonds </t>
+  </si>
+  <si>
+    <t>D-bond values selected for felony charges</t>
+  </si>
+  <si>
     <t>crime type - felonies selected</t>
   </si>
   <si>
@@ -503,46 +508,7 @@
     <t>only for violent crimes</t>
   </si>
   <si>
-    <t xml:space="preserve">Incapacitation and deterrance crime effects of detention  </t>
-  </si>
-  <si>
-    <t>Alternatives proven to be ineffecive: D-bond values selected for felony charges</t>
-  </si>
-  <si>
-    <t>Wrongful death damages Social cost of detainment (focusing on economic impact submeasure)</t>
-  </si>
-  <si>
-    <t>baseline</t>
-  </si>
-  <si>
-    <t>no. of criteria</t>
-  </si>
-  <si>
-    <t>govt_refractions</t>
-  </si>
-  <si>
-    <t>govt_health</t>
-  </si>
-  <si>
-    <t>govt_operative</t>
-  </si>
-  <si>
-    <t>soc_community</t>
-  </si>
-  <si>
-    <t>soc_crimeprev</t>
-  </si>
-  <si>
-    <t>soc_court</t>
-  </si>
-  <si>
-    <t>det_rhv</t>
-  </si>
-  <si>
-    <t>det_wtp</t>
-  </si>
-  <si>
-    <t>Scenario</t>
+    <t>Wrongful death damages Social cost of detainment (removed wtp for a human life)</t>
   </si>
 </sst>
 </file>
@@ -642,9 +608,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -950,19 +914,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{018C5E1B-70FC-CE48-BD0C-84D5CA275194}">
-  <dimension ref="A1:Q19"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="58.1640625" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="3" max="3" width="77.6640625" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.1640625" customWidth="1"/>
     <col min="11" max="11" width="16.33203125" customWidth="1"/>
     <col min="12" max="12" width="53.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="72.1640625" bestFit="1" customWidth="1"/>
@@ -1058,7 +1022,7 @@
         <v>134</v>
       </c>
       <c r="C3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1073,10 +1037,10 @@
         <v>2018</v>
       </c>
       <c r="H3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I3" s="3">
-        <v>0</v>
+        <v>75000</v>
       </c>
       <c r="J3" s="3">
         <v>133685</v>
@@ -1085,7 +1049,7 @@
         <v>75000</v>
       </c>
       <c r="L3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="M3" t="s">
         <v>108</v>
@@ -1100,7 +1064,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1123,7 +1087,7 @@
         <v>2023</v>
       </c>
       <c r="H4" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I4" s="3">
         <v>294728</v>
@@ -1135,7 +1099,7 @@
         <v>300000</v>
       </c>
       <c r="L4" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="M4" s="11" t="s">
         <v>147</v>
@@ -1158,10 +1122,10 @@
         <v>134</v>
       </c>
       <c r="C5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="s">
         <v>126</v>
@@ -1173,7 +1137,7 @@
         <v>2024</v>
       </c>
       <c r="H5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I5" s="3">
         <v>875000</v>
@@ -1185,7 +1149,7 @@
         <v>875000</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="M5" t="s">
         <v>100</v>
@@ -1470,12 +1434,6 @@
       </c>
       <c r="N13" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="19" spans="9:9" x14ac:dyDescent="0.2">
-      <c r="I19">
-        <f>+I9/I10</f>
-        <v>13217.782530564147</v>
       </c>
     </row>
   </sheetData>
@@ -1488,580 +1446,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E4AB0FE-E22E-7046-8B42-84C7BB8E6363}">
-  <dimension ref="A1:J17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.5" customWidth="1"/>
-    <col min="2" max="9" width="15.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>168</v>
-      </c>
-      <c r="B1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D1" t="s">
-        <v>165</v>
-      </c>
-      <c r="E1" t="s">
-        <v>164</v>
-      </c>
-      <c r="F1" t="s">
-        <v>163</v>
-      </c>
-      <c r="G1" t="s">
-        <v>162</v>
-      </c>
-      <c r="H1" t="s">
-        <v>161</v>
-      </c>
-      <c r="I1" t="s">
-        <v>160</v>
-      </c>
-      <c r="J1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <f>COUNTIF(B2:I2, 1)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <f>COUNTIF(B3:I3, 1)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <f>COUNTIF(B4:I4, 1)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <f>COUNTIF(B5:I5, 1)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
-      <c r="J6">
-        <f>COUNTIF(B6:I6, 1)</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
-      <c r="J7">
-        <f>COUNTIF(B7:I7, 1)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8">
-        <v>1</v>
-      </c>
-      <c r="J8">
-        <f>COUNTIF(B8:I8, 1)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>1</v>
-      </c>
-      <c r="I9">
-        <v>1</v>
-      </c>
-      <c r="J9">
-        <f>COUNTIF(B9:I9, 1)</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>1</v>
-      </c>
-      <c r="J10">
-        <f>COUNTIF(B10:I10, 1)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>1</v>
-      </c>
-      <c r="J11">
-        <f>COUNTIF(B11:I11, 1)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>1</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <v>1</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <v>1</v>
-      </c>
-      <c r="J12">
-        <f>COUNTIF(B12:I12, 1)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>0</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <v>1</v>
-      </c>
-      <c r="J13">
-        <f>COUNTIF(B13:I13, 1)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
-      </c>
-      <c r="F14">
-        <v>1</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
-        <f>COUNTIF(B14:I14, 1)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>0</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
-        <f>COUNTIF(B15:I15, 1)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16">
-        <f>COUNTIF(B16:I16, 1)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>0</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>1</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-      <c r="J17">
-        <f>COUNTIF(B17:I17, 1)</f>
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EF59096-85EC-6844-83BB-A3D9FC91749B}">
   <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2394,7 +1778,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>